<commit_message>
feat: add template serial number
</commit_message>
<xml_diff>
--- a/SHINY.xlsx
+++ b/SHINY.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luis\Documents\PROJECTS\IMPRENTA-SETH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783E97DB-3B7B-4DB6-8FFD-1162E1F4502A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC80001-6221-42AD-A599-53418E69A38E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="240" windowWidth="29040" windowHeight="16080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="360" windowWidth="14610" windowHeight="15945" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="products" sheetId="1" r:id="rId1"/>
+    <sheet name="product_templates" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="423">
   <si>
     <t>id</t>
   </si>
@@ -127,9 +127,6 @@
     <t>description</t>
   </si>
   <si>
-    <t>purchase_price</t>
-  </si>
-  <si>
     <t>final_price</t>
   </si>
   <si>
@@ -1289,13 +1286,22 @@
   </si>
   <si>
     <t>S - 822 SELLO</t>
+  </si>
+  <si>
+    <t>Trodat</t>
+  </si>
+  <si>
+    <t>template_serial_number</t>
+  </si>
+  <si>
+    <t>category</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1303,8 +1309,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1328,7 +1342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1337,6 +1351,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1552,7 +1567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="51.140625" customWidth="1"/>
@@ -1793,6 +1808,14 @@
         <v>29</v>
       </c>
     </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>420</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1801,2997 +1824,2999 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F296"/>
+  <dimension ref="A1:G298"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
     <col min="2" max="2" width="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="3" max="3" width="37" style="5" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="D1" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="5" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" t="s">
-        <v>165</v>
-      </c>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="F3" s="5">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>420</v>
-      </c>
-      <c r="C4" t="s">
-        <v>166</v>
-      </c>
-      <c r="D4" s="3"/>
-      <c r="F4">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+      <c r="D4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" t="s">
-        <v>168</v>
-      </c>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>167</v>
+      </c>
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>1</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" t="s">
-        <v>170</v>
-      </c>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s">
+        <v>169</v>
+      </c>
+      <c r="E8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>1</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>160</v>
-      </c>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s">
+        <v>159</v>
+      </c>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>1</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" t="s">
-        <v>171</v>
-      </c>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>1</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>172</v>
-      </c>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>171</v>
+      </c>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>1</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" t="s">
-        <v>173</v>
-      </c>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>1</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>174</v>
-      </c>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>173</v>
+      </c>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>1</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
-        <v>175</v>
-      </c>
-      <c r="D14" s="3"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
+        <v>174</v>
+      </c>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>1</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" t="s">
-        <v>176</v>
-      </c>
-      <c r="D15" s="3"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="D15" t="s">
+        <v>175</v>
+      </c>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>1</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" t="s">
-        <v>177</v>
-      </c>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>1</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" t="s">
-        <v>178</v>
-      </c>
-      <c r="D17" s="3"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+      <c r="D17" t="s">
+        <v>177</v>
+      </c>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>1</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" t="s">
-        <v>179</v>
-      </c>
-      <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>178</v>
+      </c>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>1</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" t="s">
-        <v>180</v>
-      </c>
-      <c r="D19" s="3"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="D19" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>1</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" t="s">
+        <v>164</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C20" t="s">
-        <v>165</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>1</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" t="s">
-        <v>181</v>
-      </c>
-      <c r="D21" s="3" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>180</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" t="s">
-        <v>166</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="D22" t="s">
+        <v>165</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>1</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" t="s">
-        <v>167</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D23" t="s">
+        <v>166</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>1</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24" t="s">
-        <v>168</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="D24" t="s">
+        <v>167</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>1</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C25" t="s">
-        <v>169</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="D25" t="s">
+        <v>168</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>1</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" t="s">
-        <v>182</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+      <c r="D26" t="s">
+        <v>181</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" t="s">
-        <v>183</v>
-      </c>
-      <c r="D27" s="3"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+      <c r="D27" t="s">
+        <v>182</v>
+      </c>
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" t="s">
-        <v>184</v>
-      </c>
-      <c r="D28" s="3"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+      <c r="D28" t="s">
+        <v>183</v>
+      </c>
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" t="s">
-        <v>185</v>
-      </c>
-      <c r="D29" s="3"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+      <c r="D29" t="s">
+        <v>184</v>
+      </c>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
-      </c>
-      <c r="C30" t="s">
-        <v>186</v>
-      </c>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="D30" t="s">
+        <v>185</v>
+      </c>
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
-      </c>
-      <c r="C31" t="s">
-        <v>187</v>
-      </c>
-      <c r="D31" s="3"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+      <c r="D31" t="s">
+        <v>186</v>
+      </c>
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
-      </c>
-      <c r="C32" t="s">
-        <v>188</v>
-      </c>
-      <c r="D32" s="3"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+      <c r="D32" t="s">
+        <v>187</v>
+      </c>
+      <c r="E32" s="3"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>1</v>
       </c>
       <c r="B33" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" t="s">
-        <v>189</v>
-      </c>
-      <c r="D33" s="3"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+      <c r="D33" t="s">
+        <v>188</v>
+      </c>
+      <c r="E33" s="3"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>1</v>
       </c>
       <c r="B34" t="s">
+        <v>65</v>
+      </c>
+      <c r="D34" t="s">
+        <v>165</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C34" t="s">
-        <v>166</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>1</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C35" t="s">
-        <v>167</v>
-      </c>
-      <c r="D35" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D35" t="s">
+        <v>166</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>1</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C36" t="s">
-        <v>168</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="D36" t="s">
+        <v>167</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>1</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C37" t="s">
-        <v>169</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="D37" t="s">
+        <v>168</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>2</v>
       </c>
       <c r="B39" t="s">
-        <v>71</v>
-      </c>
-      <c r="C39" t="s">
-        <v>166</v>
-      </c>
-      <c r="D39" s="3"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="D39" t="s">
+        <v>165</v>
+      </c>
+      <c r="E39" s="3"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>72</v>
-      </c>
-      <c r="C40" t="s">
-        <v>167</v>
-      </c>
-      <c r="D40" s="3"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+      <c r="D40" t="s">
+        <v>166</v>
+      </c>
+      <c r="E40" s="3"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>73</v>
-      </c>
-      <c r="C41" t="s">
-        <v>168</v>
-      </c>
-      <c r="D41" s="3"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="D41" t="s">
+        <v>167</v>
+      </c>
+      <c r="E41" s="3"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C43" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="D43" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
-      </c>
-      <c r="C44" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="D44" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>74</v>
-      </c>
-      <c r="C45" t="s">
-        <v>190</v>
+        <v>73</v>
       </c>
       <c r="D45" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+      <c r="E45" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>77</v>
-      </c>
-      <c r="C46" t="s">
-        <v>191</v>
+        <v>76</v>
       </c>
       <c r="D46" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+      <c r="E46" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>4</v>
       </c>
       <c r="B48" t="s">
-        <v>78</v>
-      </c>
-      <c r="C48" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+      <c r="D48" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>4</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
-      </c>
-      <c r="C49" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="D49" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>4</v>
       </c>
       <c r="B50" t="s">
-        <v>80</v>
-      </c>
-      <c r="C50" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+      <c r="D50" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>4</v>
       </c>
       <c r="B51" t="s">
-        <v>81</v>
-      </c>
-      <c r="C51" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="D51" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>4</v>
       </c>
       <c r="B52" t="s">
-        <v>82</v>
-      </c>
-      <c r="C52" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="D52" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>4</v>
       </c>
       <c r="B53" t="s">
-        <v>83</v>
-      </c>
-      <c r="C53" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+      <c r="D53" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>4</v>
       </c>
       <c r="B54" t="s">
+        <v>83</v>
+      </c>
+      <c r="D54" t="s">
+        <v>172</v>
+      </c>
+      <c r="E54" t="s">
         <v>84</v>
       </c>
-      <c r="C54" t="s">
-        <v>173</v>
-      </c>
-      <c r="D54" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>4</v>
       </c>
       <c r="B55" t="s">
-        <v>86</v>
-      </c>
-      <c r="C55" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="D55" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>4</v>
       </c>
       <c r="B56" t="s">
-        <v>87</v>
-      </c>
-      <c r="C56" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="D56" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>4</v>
       </c>
       <c r="B57" t="s">
-        <v>88</v>
-      </c>
-      <c r="C57" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+      <c r="D57" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>4</v>
       </c>
       <c r="B58" t="s">
-        <v>89</v>
-      </c>
-      <c r="C58" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="D58" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>4</v>
       </c>
       <c r="B59" t="s">
-        <v>90</v>
-      </c>
-      <c r="C59" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+      <c r="D59" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>4</v>
       </c>
       <c r="B60" t="s">
-        <v>91</v>
-      </c>
-      <c r="C60" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="D60" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>92</v>
-      </c>
-      <c r="C61" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="D61" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>5</v>
       </c>
       <c r="B63" t="s">
+        <v>92</v>
+      </c>
+      <c r="D63" t="s">
         <v>93</v>
       </c>
-      <c r="C63" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>5</v>
       </c>
       <c r="B64" t="s">
+        <v>94</v>
+      </c>
+      <c r="D64" t="s">
         <v>95</v>
       </c>
-      <c r="C64" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>5</v>
       </c>
       <c r="B65" t="s">
+        <v>96</v>
+      </c>
+      <c r="D65" t="s">
         <v>97</v>
       </c>
-      <c r="C65" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>5</v>
       </c>
       <c r="B66" t="s">
+        <v>98</v>
+      </c>
+      <c r="D66" t="s">
         <v>99</v>
       </c>
-      <c r="C66" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>5</v>
       </c>
       <c r="B67" t="s">
+        <v>100</v>
+      </c>
+      <c r="D67" t="s">
         <v>101</v>
       </c>
-      <c r="C67" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>5</v>
       </c>
       <c r="B68" t="s">
+        <v>102</v>
+      </c>
+      <c r="D68" t="s">
         <v>103</v>
       </c>
-      <c r="C68" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>5</v>
       </c>
       <c r="B69" t="s">
+        <v>104</v>
+      </c>
+      <c r="D69" t="s">
         <v>105</v>
       </c>
-      <c r="C69" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>6</v>
       </c>
       <c r="B71" t="s">
-        <v>107</v>
-      </c>
-      <c r="C71" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+      <c r="D71" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>6</v>
       </c>
       <c r="B72" t="s">
-        <v>108</v>
-      </c>
-      <c r="C72" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+      <c r="D72" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>6</v>
       </c>
       <c r="B73" t="s">
-        <v>109</v>
-      </c>
-      <c r="C73" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+      <c r="D73" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>6</v>
       </c>
       <c r="B74" t="s">
-        <v>110</v>
-      </c>
-      <c r="C74" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="D74" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>6</v>
       </c>
       <c r="B75" t="s">
+        <v>110</v>
+      </c>
+      <c r="D75" t="s">
         <v>111</v>
       </c>
-      <c r="C75" t="s">
+      <c r="E75" t="s">
         <v>112</v>
       </c>
-      <c r="D75" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>6</v>
       </c>
       <c r="B76" t="s">
-        <v>114</v>
-      </c>
-      <c r="C76" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+      <c r="D76" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>6</v>
       </c>
       <c r="B77" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>7</v>
       </c>
       <c r="B79" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>7</v>
       </c>
       <c r="B80" t="s">
-        <v>117</v>
-      </c>
-      <c r="D80" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+      <c r="E80" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>7</v>
       </c>
       <c r="B81" t="s">
-        <v>118</v>
-      </c>
-      <c r="D81" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="E81" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>7</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="D82" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="E82" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>7</v>
       </c>
       <c r="B83" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>7</v>
       </c>
       <c r="B84" t="s">
-        <v>122</v>
-      </c>
-      <c r="C84" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="D84" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="E84" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>7</v>
       </c>
       <c r="B85" t="s">
-        <v>123</v>
-      </c>
-      <c r="C85" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="D85" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="E85" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>7</v>
       </c>
       <c r="B86" t="s">
-        <v>124</v>
-      </c>
-      <c r="D86" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+      <c r="E86" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>7</v>
       </c>
       <c r="B87" t="s">
-        <v>125</v>
-      </c>
-      <c r="D87" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+      <c r="E87" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>7</v>
       </c>
       <c r="B88" t="s">
-        <v>126</v>
-      </c>
-      <c r="C88" t="s">
-        <v>193</v>
+        <v>125</v>
       </c>
       <c r="D88" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+      <c r="E88" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>7</v>
       </c>
       <c r="B89" t="s">
-        <v>127</v>
-      </c>
-      <c r="D89" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+      <c r="E89" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>7</v>
       </c>
       <c r="B90" t="s">
-        <v>128</v>
-      </c>
-      <c r="D90" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+      <c r="E90" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>7</v>
       </c>
       <c r="B91" t="s">
-        <v>129</v>
-      </c>
-      <c r="D91" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+      <c r="E91" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>7</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="D92" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+      <c r="E92" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>7</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="D93" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="E93" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>7</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="C94" t="s">
-        <v>194</v>
+        <v>131</v>
       </c>
       <c r="D94" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+      <c r="E94" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>8</v>
       </c>
       <c r="B96" t="s">
-        <v>146</v>
-      </c>
-      <c r="C96" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+      <c r="D96" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>8</v>
       </c>
       <c r="B97" t="s">
-        <v>147</v>
-      </c>
-      <c r="C97" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+      <c r="D97" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>8</v>
       </c>
       <c r="B98" t="s">
-        <v>148</v>
-      </c>
-      <c r="C98" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+      <c r="D98" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>8</v>
       </c>
       <c r="B99" t="s">
-        <v>149</v>
-      </c>
-      <c r="C99" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+      <c r="D99" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>8</v>
       </c>
       <c r="B100" t="s">
-        <v>150</v>
-      </c>
-      <c r="C100" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+      <c r="D100" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>8</v>
       </c>
       <c r="B101" t="s">
-        <v>151</v>
-      </c>
-      <c r="C101" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+      <c r="D101" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>8</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="C102" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+      <c r="D102" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>8</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C103" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+      <c r="D103" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>9</v>
       </c>
       <c r="B105" t="s">
-        <v>154</v>
-      </c>
-      <c r="C105" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+      <c r="D105" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>9</v>
       </c>
       <c r="B106" t="s">
-        <v>155</v>
-      </c>
-      <c r="C106" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+      <c r="D106" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>9</v>
       </c>
       <c r="B107" t="s">
-        <v>156</v>
-      </c>
-      <c r="C107" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="D107" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>9</v>
       </c>
       <c r="B108" t="s">
-        <v>157</v>
-      </c>
-      <c r="C108" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+      <c r="D108" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>9</v>
       </c>
       <c r="B109" t="s">
-        <v>158</v>
-      </c>
-      <c r="C109" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+      <c r="D109" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>9</v>
       </c>
       <c r="B110" t="s">
-        <v>159</v>
-      </c>
-      <c r="C110" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="D110" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="E110" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>9</v>
       </c>
       <c r="B111" t="s">
-        <v>201</v>
-      </c>
-      <c r="C111" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D111" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+      <c r="E111" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>9</v>
       </c>
       <c r="B112" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="D112" t="s">
         <v>202</v>
       </c>
-      <c r="C112" t="s">
-        <v>203</v>
-      </c>
-      <c r="D112" s="5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E112" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>10</v>
       </c>
       <c r="B114" t="s">
-        <v>207</v>
-      </c>
-      <c r="C114" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+        <v>206</v>
+      </c>
+      <c r="D114" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>10</v>
       </c>
       <c r="B115" t="s">
-        <v>208</v>
-      </c>
-      <c r="C115" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="D115" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>10</v>
       </c>
       <c r="B116" t="s">
-        <v>209</v>
-      </c>
-      <c r="C116" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+        <v>208</v>
+      </c>
+      <c r="D116" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>10</v>
       </c>
       <c r="B117" t="s">
-        <v>210</v>
-      </c>
-      <c r="C117" t="s">
+        <v>209</v>
+      </c>
+      <c r="D117" t="s">
+        <v>212</v>
+      </c>
+      <c r="E117" t="s">
         <v>213</v>
       </c>
-      <c r="D117" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>11</v>
       </c>
       <c r="B119" t="s">
-        <v>219</v>
-      </c>
-      <c r="C119" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+      <c r="D119" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>11</v>
       </c>
       <c r="B120" t="s">
-        <v>220</v>
-      </c>
-      <c r="C120" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+      <c r="D120" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>11</v>
       </c>
       <c r="B121" t="s">
-        <v>221</v>
-      </c>
-      <c r="C121" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="D121" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>11</v>
       </c>
       <c r="B122" t="s">
-        <v>222</v>
-      </c>
-      <c r="C122" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+      <c r="D122" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>11</v>
       </c>
       <c r="B123" t="s">
-        <v>223</v>
-      </c>
-      <c r="C123" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+      <c r="D123" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>11</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="C124" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D124" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E124" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>11</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="C125" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D125" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E125" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>11</v>
       </c>
       <c r="B126" t="s">
-        <v>218</v>
-      </c>
-      <c r="D126" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+      <c r="E126" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>11</v>
       </c>
       <c r="B127" t="s">
+        <v>225</v>
+      </c>
+      <c r="D127" t="s">
+        <v>202</v>
+      </c>
+      <c r="E127" t="s">
         <v>226</v>
       </c>
-      <c r="C127" t="s">
-        <v>203</v>
-      </c>
-      <c r="D127" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>11</v>
       </c>
       <c r="B128" t="s">
+        <v>227</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E128" t="s">
         <v>228</v>
       </c>
-      <c r="C128" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="D128" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>11</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="C129" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="D129" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D129" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E129" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>12</v>
       </c>
       <c r="B131" t="s">
-        <v>232</v>
-      </c>
-      <c r="C131" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+      <c r="D131" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>12</v>
       </c>
       <c r="B132" t="s">
-        <v>231</v>
-      </c>
-      <c r="C132" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+      <c r="D132" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>12</v>
       </c>
       <c r="B133" t="s">
-        <v>233</v>
-      </c>
-      <c r="C133" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+      <c r="D133" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>12</v>
       </c>
       <c r="B134" t="s">
-        <v>234</v>
-      </c>
-      <c r="C134" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+      <c r="D134" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>12</v>
       </c>
       <c r="B135" t="s">
-        <v>235</v>
-      </c>
-      <c r="C135" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+      <c r="D135" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>12</v>
       </c>
       <c r="B136" t="s">
-        <v>236</v>
-      </c>
-      <c r="C136" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+      <c r="D136" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>12</v>
       </c>
       <c r="B137" t="s">
-        <v>237</v>
-      </c>
-      <c r="C137" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="D137" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>12</v>
       </c>
       <c r="B138" t="s">
-        <v>238</v>
-      </c>
-      <c r="C138" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+        <v>237</v>
+      </c>
+      <c r="D138" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>12</v>
       </c>
       <c r="B139" t="s">
-        <v>239</v>
-      </c>
-      <c r="C139" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+        <v>238</v>
+      </c>
+      <c r="D139" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>13</v>
       </c>
       <c r="B141" t="s">
-        <v>248</v>
-      </c>
-      <c r="C141" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+        <v>247</v>
+      </c>
+      <c r="D141" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>13</v>
       </c>
       <c r="B142" t="s">
-        <v>249</v>
-      </c>
-      <c r="C142" s="5" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+        <v>248</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>13</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="C143" s="5" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+        <v>249</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>13</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="C144" s="5" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>13</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="C145" s="5" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+        <v>251</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>14</v>
       </c>
       <c r="B147" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>14</v>
       </c>
       <c r="B148" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>14</v>
       </c>
       <c r="B149" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>14</v>
       </c>
       <c r="B150" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>14</v>
       </c>
       <c r="B151" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>14</v>
       </c>
       <c r="B152" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>15</v>
       </c>
       <c r="B154" t="s">
-        <v>259</v>
-      </c>
-      <c r="C154" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="D154" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E154" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>15</v>
       </c>
       <c r="B155" t="s">
-        <v>260</v>
-      </c>
-      <c r="C155" t="s">
-        <v>268</v>
-      </c>
-      <c r="D155" s="5" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+      <c r="D155" t="s">
+        <v>267</v>
+      </c>
+      <c r="E155" s="5" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>15</v>
       </c>
       <c r="B156" t="s">
-        <v>261</v>
-      </c>
-      <c r="D156" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+        <v>260</v>
+      </c>
+      <c r="E156" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>15</v>
       </c>
       <c r="B157" t="s">
-        <v>262</v>
-      </c>
-      <c r="D157" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+      <c r="E157" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>15</v>
       </c>
       <c r="B158" t="s">
-        <v>263</v>
-      </c>
-      <c r="C158" t="s">
+        <v>262</v>
+      </c>
+      <c r="D158" t="s">
+        <v>270</v>
+      </c>
+      <c r="E158" t="s">
         <v>271</v>
       </c>
-      <c r="D158" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>15</v>
       </c>
       <c r="B159" t="s">
-        <v>264</v>
-      </c>
-      <c r="C159" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+        <v>263</v>
+      </c>
+      <c r="D159" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>15</v>
       </c>
       <c r="B160" t="s">
-        <v>265</v>
-      </c>
-      <c r="C160" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+        <v>264</v>
+      </c>
+      <c r="D160" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>15</v>
       </c>
       <c r="B161" t="s">
-        <v>277</v>
-      </c>
-      <c r="C161" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+        <v>276</v>
+      </c>
+      <c r="D161" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>15</v>
       </c>
       <c r="B162" t="s">
-        <v>278</v>
-      </c>
-      <c r="C162" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+        <v>277</v>
+      </c>
+      <c r="D162" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>16</v>
       </c>
       <c r="B164" t="s">
-        <v>282</v>
-      </c>
-      <c r="C164" t="s">
-        <v>134</v>
+        <v>281</v>
       </c>
       <c r="D164" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="E164" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>16</v>
       </c>
       <c r="B165" t="s">
-        <v>283</v>
-      </c>
-      <c r="C165" s="5" t="s">
-        <v>133</v>
+        <v>282</v>
       </c>
       <c r="D165" s="5" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="E165" s="5" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>16</v>
       </c>
       <c r="B166" t="s">
-        <v>284</v>
-      </c>
-      <c r="C166" s="5" t="s">
-        <v>203</v>
+        <v>283</v>
       </c>
       <c r="D166" s="5" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+      <c r="E166" s="5" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>16</v>
       </c>
       <c r="B167" t="s">
-        <v>285</v>
-      </c>
-      <c r="C167" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D167" s="5" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E167" s="5" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>16</v>
       </c>
       <c r="B168" t="s">
-        <v>286</v>
-      </c>
-      <c r="C168" s="5" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="D168" s="5" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+      <c r="E168" s="5" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>17</v>
       </c>
       <c r="B170" t="s">
-        <v>287</v>
-      </c>
-      <c r="C170" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+      <c r="D170" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>17</v>
       </c>
       <c r="B171" t="s">
-        <v>288</v>
-      </c>
-      <c r="C171" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+        <v>287</v>
+      </c>
+      <c r="D171" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>17</v>
       </c>
       <c r="B172" t="s">
-        <v>289</v>
-      </c>
-      <c r="C172" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="D172" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>17</v>
       </c>
       <c r="B173" t="s">
-        <v>290</v>
-      </c>
-      <c r="C173" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+        <v>289</v>
+      </c>
+      <c r="D173" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>17</v>
       </c>
       <c r="B174" t="s">
-        <v>291</v>
-      </c>
-      <c r="C174" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+        <v>290</v>
+      </c>
+      <c r="D174" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>17</v>
       </c>
       <c r="B175" t="s">
-        <v>292</v>
-      </c>
-      <c r="D175" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+        <v>291</v>
+      </c>
+      <c r="E175" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>18</v>
       </c>
       <c r="B177" t="s">
-        <v>298</v>
-      </c>
-      <c r="C177" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+        <v>297</v>
+      </c>
+      <c r="D177" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>18</v>
       </c>
       <c r="B178" t="s">
-        <v>299</v>
-      </c>
-      <c r="C178" s="5" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+        <v>298</v>
+      </c>
+      <c r="D178" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>18</v>
       </c>
       <c r="B179" t="s">
-        <v>300</v>
-      </c>
-      <c r="C179" s="5" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+        <v>299</v>
+      </c>
+      <c r="D179" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>19</v>
       </c>
       <c r="B181" t="s">
-        <v>301</v>
-      </c>
-      <c r="C181" t="s">
-        <v>134</v>
+        <v>300</v>
       </c>
       <c r="D181" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="E181" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>19</v>
       </c>
       <c r="B182" t="s">
-        <v>302</v>
-      </c>
-      <c r="C182" t="s">
-        <v>134</v>
+        <v>301</v>
       </c>
       <c r="D182" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+      <c r="E182" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>19</v>
       </c>
       <c r="B183" t="s">
-        <v>303</v>
-      </c>
-      <c r="C183" t="s">
-        <v>133</v>
+        <v>302</v>
       </c>
       <c r="D183" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="E183" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>19</v>
       </c>
       <c r="B184" t="s">
-        <v>304</v>
-      </c>
-      <c r="C184" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="D184" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+        <v>303</v>
+      </c>
+      <c r="D184" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E184" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>19</v>
       </c>
       <c r="B185" t="s">
-        <v>305</v>
-      </c>
-      <c r="C185" t="s">
-        <v>203</v>
+        <v>304</v>
       </c>
       <c r="D185" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+      <c r="E185" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>19</v>
       </c>
       <c r="B186" t="s">
-        <v>306</v>
-      </c>
-      <c r="C186" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="D186" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+        <v>305</v>
+      </c>
+      <c r="D186" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E186" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>19</v>
       </c>
       <c r="B187" t="s">
-        <v>307</v>
-      </c>
-      <c r="C187" t="s">
-        <v>281</v>
+        <v>306</v>
       </c>
       <c r="D187" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+      <c r="E187" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>19</v>
       </c>
       <c r="B188" t="s">
-        <v>308</v>
-      </c>
-      <c r="C188" t="s">
-        <v>281</v>
+        <v>307</v>
       </c>
       <c r="D188" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+      <c r="E188" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>20</v>
       </c>
       <c r="B190" t="s">
-        <v>312</v>
-      </c>
-      <c r="C190" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D190" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+        <v>316</v>
+      </c>
+      <c r="E190" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>20</v>
       </c>
       <c r="B191" t="s">
-        <v>313</v>
-      </c>
-      <c r="C191" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="D191" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+        <v>317</v>
+      </c>
+      <c r="E191" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>20</v>
       </c>
       <c r="B192" t="s">
-        <v>314</v>
-      </c>
-      <c r="C192" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D192" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+        <v>318</v>
+      </c>
+      <c r="E192" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="2">
         <v>20</v>
       </c>
       <c r="B193" t="s">
-        <v>315</v>
-      </c>
-      <c r="C193" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="D193" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+        <v>318</v>
+      </c>
+      <c r="E193" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
         <v>20</v>
       </c>
       <c r="B194" t="s">
-        <v>316</v>
-      </c>
-      <c r="C194" t="s">
-        <v>203</v>
+        <v>315</v>
       </c>
       <c r="D194" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+      <c r="E194" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
         <v>21</v>
       </c>
       <c r="B196" t="s">
-        <v>321</v>
-      </c>
-      <c r="D196" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+        <v>320</v>
+      </c>
+      <c r="E196" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>21</v>
       </c>
       <c r="B197" t="s">
-        <v>322</v>
-      </c>
-      <c r="D197" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+        <v>321</v>
+      </c>
+      <c r="E197" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
         <v>21</v>
       </c>
       <c r="B198" t="s">
-        <v>323</v>
-      </c>
-      <c r="D198" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+        <v>322</v>
+      </c>
+      <c r="E198" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="2">
         <v>21</v>
       </c>
       <c r="B199" t="s">
-        <v>324</v>
-      </c>
-      <c r="D199" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+        <v>323</v>
+      </c>
+      <c r="E199" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="2">
         <v>22</v>
       </c>
       <c r="B201" t="s">
-        <v>330</v>
-      </c>
-      <c r="C201" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+        <v>329</v>
+      </c>
+      <c r="D201" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="2">
         <v>22</v>
       </c>
       <c r="B202" t="s">
-        <v>329</v>
-      </c>
-      <c r="C202" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+        <v>328</v>
+      </c>
+      <c r="D202" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="2">
         <v>23</v>
       </c>
       <c r="B204" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="2">
         <v>23</v>
       </c>
       <c r="B205" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="2">
         <v>23</v>
       </c>
       <c r="B206" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="2">
         <v>24</v>
       </c>
       <c r="B208" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="2">
         <v>24</v>
       </c>
       <c r="B209" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="2">
         <v>24</v>
       </c>
       <c r="B210" t="s">
-        <v>337</v>
-      </c>
-      <c r="D210" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+        <v>336</v>
+      </c>
+      <c r="E210" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="2">
         <v>24</v>
       </c>
       <c r="B211" t="s">
-        <v>338</v>
-      </c>
-      <c r="D211" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+        <v>337</v>
+      </c>
+      <c r="E211" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="2">
         <v>24</v>
       </c>
       <c r="B212" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="2">
         <v>24</v>
       </c>
       <c r="B213" t="s">
-        <v>339</v>
-      </c>
-      <c r="D213" s="5" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+        <v>338</v>
+      </c>
+      <c r="E213" s="5" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="2">
         <v>24</v>
       </c>
       <c r="B214" t="s">
-        <v>339</v>
-      </c>
-      <c r="D214" s="5" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+        <v>338</v>
+      </c>
+      <c r="E214" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="2">
         <v>24</v>
       </c>
       <c r="B215" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="2">
         <v>24</v>
       </c>
       <c r="B216" t="s">
-        <v>340</v>
-      </c>
-      <c r="D216" s="5" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+      <c r="E216" s="5" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="2">
         <v>24</v>
       </c>
       <c r="B217" t="s">
-        <v>341</v>
-      </c>
-      <c r="D217" s="5" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+      <c r="E217" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="2">
         <v>24</v>
       </c>
       <c r="B218" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="2">
         <v>24</v>
       </c>
       <c r="B219" t="s">
-        <v>342</v>
-      </c>
-      <c r="D219" s="5" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+        <v>341</v>
+      </c>
+      <c r="E219" s="5" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="2">
         <v>24</v>
       </c>
       <c r="B220" t="s">
-        <v>342</v>
-      </c>
-      <c r="D220" s="5" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+        <v>341</v>
+      </c>
+      <c r="E220" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="2">
         <v>24</v>
       </c>
       <c r="B221" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="2">
         <v>24</v>
       </c>
       <c r="B222" t="s">
-        <v>344</v>
-      </c>
-      <c r="D222" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+        <v>343</v>
+      </c>
+      <c r="E222" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="2">
         <v>25</v>
       </c>
       <c r="B224" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="2">
         <v>25</v>
       </c>
       <c r="B225" t="s">
-        <v>348</v>
-      </c>
-      <c r="D225" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E225" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="2">
         <v>25</v>
       </c>
       <c r="B226" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="2">
         <v>25</v>
       </c>
       <c r="B227" t="s">
-        <v>349</v>
-      </c>
-      <c r="D227" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+        <v>348</v>
+      </c>
+      <c r="E227" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="2">
         <v>25</v>
       </c>
       <c r="B228" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="2">
         <v>25</v>
       </c>
       <c r="B229" t="s">
-        <v>350</v>
-      </c>
-      <c r="D229" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+      <c r="E229" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="2">
         <v>25</v>
       </c>
       <c r="B230" t="s">
-        <v>350</v>
-      </c>
-      <c r="D230" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+      <c r="E230" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="2">
         <v>25</v>
       </c>
       <c r="B231" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="2">
         <v>25</v>
       </c>
       <c r="B232" t="s">
-        <v>351</v>
-      </c>
-      <c r="D232" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+      <c r="E232" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="2">
         <v>25</v>
       </c>
       <c r="B233" t="s">
-        <v>351</v>
-      </c>
-      <c r="D233" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+      <c r="E233" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="2">
         <v>25</v>
       </c>
       <c r="B234" t="s">
-        <v>351</v>
-      </c>
-      <c r="D234" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+      <c r="E234" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="2">
         <v>25</v>
       </c>
       <c r="B235" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="2">
         <v>25</v>
       </c>
       <c r="B236" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="2">
         <v>25</v>
       </c>
       <c r="B237" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="2">
         <v>25</v>
       </c>
       <c r="B238" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="2">
         <v>25</v>
       </c>
       <c r="B239" t="s">
-        <v>355</v>
-      </c>
-      <c r="D239" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+      <c r="E239" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="2">
         <v>25</v>
       </c>
       <c r="B240" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="2">
         <v>25</v>
       </c>
       <c r="B241" t="s">
-        <v>356</v>
-      </c>
-      <c r="D241" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+      <c r="E241" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="2">
         <v>25</v>
       </c>
       <c r="B242" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="2">
         <v>25</v>
       </c>
       <c r="B243" t="s">
-        <v>357</v>
-      </c>
-      <c r="D243" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+        <v>356</v>
+      </c>
+      <c r="E243" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="2">
         <v>25</v>
       </c>
       <c r="B244" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="2">
         <v>25</v>
       </c>
       <c r="B245" t="s">
-        <v>358</v>
-      </c>
-      <c r="D245" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+        <v>357</v>
+      </c>
+      <c r="E245" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="2">
         <v>25</v>
       </c>
       <c r="B246" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="2">
         <v>25</v>
       </c>
       <c r="B247" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="2">
         <v>25</v>
       </c>
       <c r="B248" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="2">
         <v>26</v>
       </c>
       <c r="B250" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="2">
         <v>26</v>
       </c>
       <c r="B251" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="2">
         <v>26</v>
       </c>
       <c r="B252" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="2">
         <v>26</v>
       </c>
       <c r="B253" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="2">
         <v>26</v>
       </c>
       <c r="B254" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="2">
         <v>26</v>
       </c>
       <c r="B255" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="2">
         <v>26</v>
       </c>
       <c r="B256" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="2">
         <v>26</v>
       </c>
       <c r="B257" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="2">
         <v>26</v>
       </c>
       <c r="B258" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="2">
         <v>26</v>
       </c>
       <c r="B259" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="2">
         <v>26</v>
       </c>
       <c r="B260" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="2">
         <v>26</v>
       </c>
       <c r="B261" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="2">
         <v>26</v>
       </c>
       <c r="B262" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="2">
         <v>26</v>
       </c>
       <c r="B263" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="2">
         <v>26</v>
       </c>
       <c r="B264" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="2">
         <v>26</v>
       </c>
       <c r="B265" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="2">
         <v>26</v>
       </c>
       <c r="B266" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="2">
         <v>26</v>
       </c>
       <c r="B267" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="2">
         <v>26</v>
       </c>
       <c r="B268" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="2">
         <v>26</v>
       </c>
       <c r="B269" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="2">
         <v>26</v>
       </c>
       <c r="B270" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="D270" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
+        <v>379</v>
+      </c>
+      <c r="E270" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="2">
         <v>26</v>
       </c>
       <c r="B271" t="s">
-        <v>382</v>
-      </c>
-      <c r="D271" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+      <c r="E271" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="2">
         <v>26</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="D272" s="5" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+      <c r="E272" s="5" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="2">
         <v>26</v>
       </c>
       <c r="B273" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="2">
         <v>26</v>
       </c>
       <c r="B274" t="s">
-        <v>387</v>
-      </c>
-      <c r="D274" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="275" spans="1:4" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+      <c r="E274" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="2">
         <v>26</v>
       </c>
       <c r="B275" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="276" spans="1:4" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="2">
         <v>26</v>
       </c>
       <c r="B276" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="277" spans="1:4" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="2">
         <v>26</v>
       </c>
       <c r="B277" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="278" spans="1:4" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="2">
         <v>26</v>
       </c>
       <c r="B278" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="279" spans="1:4" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="2">
         <v>26</v>
       </c>
       <c r="B279" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="280" spans="1:4" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="2">
         <v>26</v>
       </c>
       <c r="B280" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="281" spans="1:4" x14ac:dyDescent="0.25">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="2">
         <v>26</v>
       </c>
       <c r="B281" t="s">
-        <v>395</v>
-      </c>
-      <c r="D281" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+      <c r="E281" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="2">
         <v>26</v>
       </c>
       <c r="B282" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" s="2">
         <v>26</v>
       </c>
       <c r="B283" t="s">
+        <v>396</v>
+      </c>
+      <c r="E283" t="s">
         <v>397</v>
       </c>
-      <c r="D283" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="284" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="2">
         <v>26</v>
       </c>
       <c r="B284" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="285" spans="1:4" x14ac:dyDescent="0.25">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" s="2">
         <v>26</v>
       </c>
       <c r="B285" t="s">
-        <v>400</v>
-      </c>
-      <c r="D285" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="286" spans="1:4" x14ac:dyDescent="0.25">
+        <v>399</v>
+      </c>
+      <c r="E285" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" s="2">
         <v>26</v>
       </c>
       <c r="B286" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="287" spans="1:4" x14ac:dyDescent="0.25">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="2">
         <v>26</v>
       </c>
       <c r="B287" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="2">
         <v>27</v>
       </c>
       <c r="B289" t="s">
-        <v>403</v>
-      </c>
-      <c r="C289" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="D289" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="290" spans="1:4" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+      <c r="E289" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" s="2">
         <v>27</v>
       </c>
       <c r="B290" t="s">
-        <v>404</v>
-      </c>
-      <c r="C290" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="D290" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="291" spans="1:4" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+      <c r="E290" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="2">
         <v>27</v>
       </c>
       <c r="B291" t="s">
-        <v>405</v>
-      </c>
-      <c r="C291" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="D291" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="292" spans="1:4" x14ac:dyDescent="0.25">
+        <v>411</v>
+      </c>
+      <c r="E291" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="2">
         <v>27</v>
       </c>
       <c r="B292" t="s">
-        <v>406</v>
-      </c>
-      <c r="C292" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="D292" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="293" spans="1:4" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+      <c r="D292" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="E292" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="2">
         <v>27</v>
       </c>
       <c r="B293" t="s">
+        <v>406</v>
+      </c>
+      <c r="D293" t="s">
+        <v>412</v>
+      </c>
+      <c r="E293" t="s">
         <v>407</v>
       </c>
-      <c r="C293" t="s">
-        <v>413</v>
-      </c>
-      <c r="D293" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="2">
         <v>28</v>
       </c>
       <c r="B295" t="s">
-        <v>414</v>
-      </c>
-      <c r="C295" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D295" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
+        <v>415</v>
+      </c>
+      <c r="E295" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="2">
         <v>28</v>
       </c>
       <c r="B296" t="s">
-        <v>415</v>
-      </c>
-      <c r="C296" t="s">
-        <v>417</v>
+        <v>414</v>
+      </c>
+      <c r="D296" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A298" s="2">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>